<commit_message>
feat(csv): 10-column observation schema + phase1 default + multi -p merge
</commit_message>
<xml_diff>
--- a/options.xlsx
+++ b/options.xlsx
@@ -60,21 +60,21 @@
     <t>-sS</t>
   </si>
   <si>
+    <t>TCP 스캔 타입</t>
+  </si>
+  <si>
+    <t>Half-open TCP SYN 스캔 (-sS). raw socket 권한(=관리자) 필요. 타겟에 완전한 TCP 연결을 안 만들어 stealth, 빠름. 권한 없으면 nmap이 자동으로 -sT 로 폴백.</t>
+  </si>
+  <si>
+    <t>Connect</t>
+  </si>
+  <si>
+    <t>-sT</t>
+  </si>
+  <si>
     <t>0</t>
   </si>
   <si>
-    <t>TCP 스캔 타입</t>
-  </si>
-  <si>
-    <t>Half-open TCP SYN 스캔 (-sS). raw socket 권한(=관리자) 필요. 타겟에 완전한 TCP 연결을 안 만들어 stealth, 빠름. 권한 없으면 nmap이 자동으로 -sT 로 폴백.</t>
-  </si>
-  <si>
-    <t>Connect</t>
-  </si>
-  <si>
-    <t>-sT</t>
-  </si>
-  <si>
     <t>정상 TCP 3-way handshake 완성 (-sT). 일반 사용자 권한으로 가능. 타겟 로그에 connect 흔적이 더 남고 -sS 보다 약간 느림.</t>
   </si>
   <si>
@@ -174,10 +174,10 @@
     <t>UDP 주요 포트 스캔</t>
   </si>
   <si>
-    <t>-sU -p U:7,53,67,68,69,123,135,137,138,139,161,162,500,514,520,1900,4500,5060,5353,11211</t>
-  </si>
-  <si>
-    <t>UDP 스캔 + 자주 쓰이는 22 포트만. UDP 는 RST 응답이 없어 매우 느림. 포트를 좁힐수록 시간 단축. SNMP, NetBIOS, IKE, SIP 등 식별.</t>
+    <t>-sU -p U:7,53,67,68,69,88,123,135,137,138,139,161,162,389,400,500,514,520,623,1900,2049,4500,5060,5353,5355,11211</t>
+  </si>
+  <si>
+    <t>UDP 스캔 + 자주 쓰이는 26 포트 (DNS, NetBIOS, SNMP, Kerberos, IKE, SIP, NTP, NFS, mDNS 등). UDP 는 RST 응답 없어 느림. -p T:... 와 합쳐 단일 -p T:...,U:... 로 출력.</t>
   </si>
   <si>
     <t>TCP 모든 포트 (1-65535)</t>
@@ -186,7 +186,7 @@
     <t>-p T:1-65535</t>
   </si>
   <si>
-    <t>TCP 65535 포트 전부 SYN 보냄. T4 기준 호스트당 5~15분. 전수 점검용. 시간 많이 걸려 일반 점검에선 자주 쓰는 포트만 권장.</t>
+    <t>TCP 65535 포트 전부 SYN 보냄. T4 기준 호스트당 5~15분. 전수 점검용 (phase1 기본).</t>
   </si>
   <si>
     <t>서비스 버전 식별</t>
@@ -249,7 +249,7 @@
     <t>--min-hostgroup 64</t>
   </si>
   <si>
-    <t>한 번에 64개 호스트를 병렬로 스캔. /24 같은 큰 대역 스캔 시 처리량 증가. 메모리/대역폭 더 사용.</t>
+    <t>한 번에 64개 호스트를 병렬로 스캔. /24 같은 큰 대역 스캔 시 처리량 증가.</t>
   </si>
   <si>
     <t>동시 처리 100</t>
@@ -258,7 +258,7 @@
     <t>--max-parallelism 100</t>
   </si>
   <si>
-    <t>동시 in-flight probe 100개까지. 빠른 네트워크에서 처리량 증가. 너무 높으면 IDS 트리거/패킷 손실.</t>
+    <t>동시 in-flight probe 100개까지. 빠른 네트워크에서 처리량 증가.</t>
   </si>
   <si>
     <t>Aggressive 모드 (-A)</t>
@@ -267,7 +267,7 @@
     <t>-A</t>
   </si>
   <si>
-    <t>공격적 옵션 묶음 (-O OS 식별 + -sV + -sC default NSE + --traceroute). 매우 빠르게 정보 모음. 대신 흔적 많아 stealth 불가.</t>
+    <t>공격적 옵션 묶음 (-O OS 식별 + -sV + -sC default NSE + --traceroute). phase1 default 에는 미포함.</t>
   </si>
   <si>
     <t>진행 stats 1분마다 출력 (--stats-every 1m)</t>
@@ -294,7 +294,7 @@
     <t>--script ssl-cert</t>
   </si>
   <si>
-    <t>TLS 인증서의 CN, SAN(Subject Alternative Name), Issuer, Validity 추출. 점검에서 가장 큰 정보 노출 NSE 중 하나 — 인증서가 내부 호스트명을 노출시킴.</t>
+    <t>TLS 인증서의 CN, SAN(Subject Alternative Name), Issuer, Validity 추출. 인증서가 내부 호스트명을 노출시키므로 점검 핵심.</t>
   </si>
   <si>
     <t>TLS cipher / ALPN 식별</t>
@@ -318,28 +318,28 @@
     <t>SMB 식별</t>
   </si>
   <si>
-    <t>--script nbstat,smb-os-discovery,smb-protocols,smb-security-mode</t>
-  </si>
-  <si>
-    <t>Windows OS 버전, 도메인, NetBIOS 이름, SMB 버전, 보안 모드 (signing 강제 여부). AD 환경 점검 필수.</t>
-  </si>
-  <si>
-    <t>DBMS 식별</t>
-  </si>
-  <si>
-    <t>--script ms-sql-info,mysql-info,oracle-tns-version,mongodb-info,redis-info</t>
-  </si>
-  <si>
-    <t>MS-SQL/MySQL/Oracle/MongoDB/Redis 버전과 일부 설정. 인증 안 된 DB 노출 여부도 식별.</t>
-  </si>
-  <si>
-    <t>RDP/VNC/AJP 식별</t>
-  </si>
-  <si>
-    <t>--script rdp-ntlm-info,rdp-enum-encryption,vnc-info,ajp-headers</t>
-  </si>
-  <si>
-    <t>RDP NTLM 정보 (호스트명/도메인), RDP 암호화 모드, VNC 인증, AJP 헤더. 원격 접속 서비스 점검.</t>
+    <t>--script nbstat,smb-os-discovery,smb-protocols</t>
+  </si>
+  <si>
+    <t>Windows OS 버전, 도메인, NetBIOS 이름, SMB 버전. AD 환경 점검 필수. (phase1: smb-security-mode 제외)</t>
+  </si>
+  <si>
+    <t>DBMS 식별 (MS-SQL / Oracle)</t>
+  </si>
+  <si>
+    <t>--script ms-sql-info,oracle-tns-version</t>
+  </si>
+  <si>
+    <t>MS-SQL Server, Oracle TNS 버전 정보. (phase1: mysql/mongodb/redis 별도 NSE 미포함)</t>
+  </si>
+  <si>
+    <t>RDP 식별</t>
+  </si>
+  <si>
+    <t>--script rdp-ntlm-info</t>
+  </si>
+  <si>
+    <t>RDP NTLM 정보 (호스트명/도메인). (phase1: rdp-enum-encryption / vnc-info / ajp-headers 미포함)</t>
   </si>
   <si>
     <t>UDP 응용 식별 (SNMP/IKE/SIP/NTP)</t>
@@ -348,7 +348,7 @@
     <t>--script snmp-info,ike-version,sip-methods,ntp-info</t>
   </si>
   <si>
-    <t>SNMP community / OID 정보, IKE/IPSec 버전, SIP 지원 method, NTP 서버 정보. UDP 스캔과 함께 써야 의미.</t>
+    <t>SNMP community / OID, IKE/IPsec 버전, SIP 지원 method, NTP 서버 정보. UDP 스캔(-sU)과 함께 써야 의미.</t>
   </si>
   <si>
     <t>RPC 정보</t>
@@ -366,16 +366,16 @@
     <t>--script ldap-rootdse</t>
   </si>
   <si>
-    <t>LDAP root DSE 정보 추출. AD/LDAP 서버 도메인, naming context, 지원 컨트롤 등.</t>
+    <t>LDAP root DSE 정보 추출. AD/LDAP 서버 도메인, naming context. (phase1 default: 0)</t>
   </si>
   <si>
     <t>raw 응답 캡처 (식별 실패 포트)</t>
   </si>
   <si>
-    <t>--script fingerprint-strings,banner</t>
-  </si>
-  <si>
-    <t>식별 실패한 포트의 원본 응답 바이트 캡쳐. unknown 서비스를 수동 분석할 때 필수. 결과 파일 커짐.</t>
+    <t>--script fingerprint-strings</t>
+  </si>
+  <si>
+    <t>식별 실패한 포트의 원본 응답 바이트 캡쳐 (fingerprint-strings). unknown 서비스 수동 분석 필수.</t>
   </si>
 </sst>
 </file>
@@ -482,27 +482,27 @@
         <v>14</v>
       </c>
       <c r="C4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>16</v>
-      </c>
-      <c r="E4" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E5" t="s">
         <v>20</v>
@@ -516,10 +516,10 @@
         <v>22</v>
       </c>
       <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" t="s">
         <v>15</v>
-      </c>
-      <c r="D6" t="s">
-        <v>16</v>
       </c>
       <c r="E6" t="s">
         <v>23</v>
@@ -533,10 +533,10 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
         <v>15</v>
-      </c>
-      <c r="D7" t="s">
-        <v>16</v>
       </c>
       <c r="E7" t="s">
         <v>26</v>
@@ -550,10 +550,10 @@
         <v>28</v>
       </c>
       <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
         <v>15</v>
-      </c>
-      <c r="D8" t="s">
-        <v>16</v>
       </c>
       <c r="E8" t="s">
         <v>29</v>
@@ -567,10 +567,10 @@
         <v>31</v>
       </c>
       <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
         <v>15</v>
-      </c>
-      <c r="D9" t="s">
-        <v>16</v>
       </c>
       <c r="E9" t="s">
         <v>32</v>
@@ -584,7 +584,7 @@
         <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D10" t="s">
         <v>35</v>
@@ -601,7 +601,7 @@
         <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
         <v>35</v>
@@ -618,7 +618,7 @@
         <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D12" t="s">
         <v>35</v>
@@ -635,7 +635,7 @@
         <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D13" t="s">
         <v>35</v>
@@ -669,7 +669,7 @@
         <v>50</v>
       </c>
       <c r="C15" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D15" t="s">
         <v>35</v>
@@ -686,7 +686,7 @@
         <v>53</v>
       </c>
       <c r="C16" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D16" t="s">
         <v>8</v>
@@ -703,7 +703,7 @@
         <v>56</v>
       </c>
       <c r="C17" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D17" t="s">
         <v>8</v>
@@ -805,7 +805,7 @@
         <v>74</v>
       </c>
       <c r="C23" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D23" t="s">
         <v>8</v>
@@ -822,7 +822,7 @@
         <v>77</v>
       </c>
       <c r="C24" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D24" t="s">
         <v>8</v>
@@ -839,7 +839,7 @@
         <v>80</v>
       </c>
       <c r="C25" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D25" t="s">
         <v>8</v>
@@ -856,7 +856,7 @@
         <v>83</v>
       </c>
       <c r="C26" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D26" t="s">
         <v>8</v>
@@ -890,7 +890,7 @@
         <v>89</v>
       </c>
       <c r="C28" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D28" t="s">
         <v>8</v>
@@ -907,7 +907,7 @@
         <v>92</v>
       </c>
       <c r="C29" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D29" t="s">
         <v>8</v>
@@ -924,7 +924,7 @@
         <v>95</v>
       </c>
       <c r="C30" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D30" t="s">
         <v>8</v>
@@ -941,7 +941,7 @@
         <v>98</v>
       </c>
       <c r="C31" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D31" t="s">
         <v>8</v>
@@ -958,7 +958,7 @@
         <v>101</v>
       </c>
       <c r="C32" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D32" t="s">
         <v>8</v>
@@ -975,7 +975,7 @@
         <v>104</v>
       </c>
       <c r="C33" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D33" t="s">
         <v>8</v>
@@ -992,7 +992,7 @@
         <v>107</v>
       </c>
       <c r="C34" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D34" t="s">
         <v>8</v>
@@ -1009,7 +1009,7 @@
         <v>110</v>
       </c>
       <c r="C35" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D35" t="s">
         <v>8</v>
@@ -1026,7 +1026,7 @@
         <v>113</v>
       </c>
       <c r="C36" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D36" t="s">
         <v>8</v>
@@ -1043,7 +1043,7 @@
         <v>116</v>
       </c>
       <c r="C37" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D37" t="s">
         <v>8</v>
@@ -1060,7 +1060,7 @@
         <v>119</v>
       </c>
       <c r="C38" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D38" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
feat: harden Excel reporting workflow
</commit_message>
<xml_diff>
--- a/options.xlsx
+++ b/options.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="139">
   <si>
     <t>스캔 옵션</t>
   </si>
@@ -376,52 +376,116 @@
   </si>
   <si>
     <t>식별 실패한 포트의 원본 응답 바이트 캡쳐 (fingerprint-strings). unknown 서비스 수동 분석 필수.</t>
+  </si>
+  <si>
+    <t>OS 탐지 (-O)</t>
+  </si>
+  <si>
+    <t>-O</t>
+  </si>
+  <si>
+    <t>FTP 익명 로그인 / 시스템 식별</t>
+  </si>
+  <si>
+    <t>--script ftp-anon,ftp-syst</t>
+  </si>
+  <si>
+    <t>Telnet 암호화 지원 식별</t>
+  </si>
+  <si>
+    <t>--script telnet-encryption</t>
+  </si>
+  <si>
+    <t>DNS 재귀 응답 / 서버 식별 (NSID)</t>
+  </si>
+  <si>
+    <t>--script dns-recursion,dns-nsid</t>
+  </si>
+  <si>
+    <t>VNC 식별 (버전 / 보안 타입 / 타이틀)</t>
+  </si>
+  <si>
+    <t>--script vnc-info,vnc-title</t>
+  </si>
+  <si>
+    <t>NTP monlist (DDoS amp 위험)</t>
+  </si>
+  <si>
+    <t>--script ntp-monlist</t>
+  </si>
+  <si>
+    <t>일반 배너 캡처 (Rlogin / RSH 등 보완)</t>
+  </si>
+  <si>
+    <t>--script banner</t>
+  </si>
+  <si>
+    <t>SSH 인증 방식 / 알고리즘 (선택)</t>
+  </si>
+  <si>
+    <t>--script ssh-auth-methods,ssh2-enum-algos</t>
+  </si>
+  <si>
+    <t>SNMP sysDescr (선택)</t>
+  </si>
+  <si>
+    <t>--script snmp-sysdescr</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="1">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="2" width="64" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="80" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s" s="1">
@@ -1069,6 +1133,159 @@
         <v>120</v>
       </c>
     </row>
+    <row r="39" spans="1:5">
+      <c r="A39" t="s">
+        <v>121</v>
+      </c>
+      <c r="B39" t="s">
+        <v>122</v>
+      </c>
+      <c r="C39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" t="s">
+        <v>123</v>
+      </c>
+      <c r="B40" t="s">
+        <v>124</v>
+      </c>
+      <c r="C40" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" t="s">
+        <v>125</v>
+      </c>
+      <c r="B41" t="s">
+        <v>126</v>
+      </c>
+      <c r="C41" t="s">
+        <v>19</v>
+      </c>
+      <c r="D41" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" t="s">
+        <v>127</v>
+      </c>
+      <c r="B42" t="s">
+        <v>128</v>
+      </c>
+      <c r="C42" t="s">
+        <v>19</v>
+      </c>
+      <c r="D42" t="s">
+        <v>8</v>
+      </c>
+      <c r="E42" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" t="s">
+        <v>129</v>
+      </c>
+      <c r="B43" t="s">
+        <v>130</v>
+      </c>
+      <c r="C43" t="s">
+        <v>19</v>
+      </c>
+      <c r="D43" t="s">
+        <v>8</v>
+      </c>
+      <c r="E43" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" t="s">
+        <v>131</v>
+      </c>
+      <c r="B44" t="s">
+        <v>132</v>
+      </c>
+      <c r="C44" t="s">
+        <v>19</v>
+      </c>
+      <c r="D44" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" t="s">
+        <v>133</v>
+      </c>
+      <c r="B45" t="s">
+        <v>134</v>
+      </c>
+      <c r="C45" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" t="s">
+        <v>8</v>
+      </c>
+      <c r="E45" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" t="s">
+        <v>135</v>
+      </c>
+      <c r="B46" t="s">
+        <v>136</v>
+      </c>
+      <c r="C46" t="s">
+        <v>19</v>
+      </c>
+      <c r="D46" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" t="s">
+        <v>137</v>
+      </c>
+      <c r="B47" t="s">
+        <v>138</v>
+      </c>
+      <c r="C47" t="s">
+        <v>19</v>
+      </c>
+      <c r="D47" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>